<commit_message>
Improve plant naming: expand abbreviated genera, fix typos, standardize cultivar formatting; rebuild catalog
</commit_message>
<xml_diff>
--- a/catalog/Plant_Catalog_2026.xlsx
+++ b/catalog/Plant_Catalog_2026.xlsx
@@ -448,8 +448,8 @@
   <dimension ref="A1:E290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -485,7 +485,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aglaonema 'A024'</t>
+          <t>Aglaonema 'A019'</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -506,7 +506,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aglaonema A019</t>
+          <t>Aglaonema 'A024'</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Aglaonema A029</t>
+          <t>Aglaonema 'A029'</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -548,7 +548,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Aglaonema Red Angel</t>
+          <t>Aglaonema 'Red Vein'</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -560,16 +560,16 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>780</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Aglaonema sp.</t>
+          <t>Aglaonema Red Angel</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -581,16 +581,16 @@
         <v>1</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>520</v>
+        <v>780</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Aglonema red vein</t>
+          <t>Aglaonema sp.</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -602,10 +602,10 @@
         <v>1</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>156</v>
+        <v>520</v>
       </c>
     </row>
     <row r="8">
@@ -695,7 +695,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Alocasia 'Jacklyn'</t>
+          <t>Alocasia 'Heart Balloon' variegata</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -707,16 +707,16 @@
         <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>6</v>
+        <v>130</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>312</v>
+        <v>6760</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Alocasia 'Ninja'</t>
+          <t>Alocasia 'Helian'</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -727,17 +727,13 @@
       <c r="C13" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>3380</v>
-      </c>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Alocasia 'Pink Dragon'</t>
+          <t>Alocasia 'Jacklyn'</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -749,16 +745,16 @@
         <v>1</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>5200</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Alocasia 'Portora'</t>
+          <t>Alocasia 'Ninja'</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -779,7 +775,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Alocasia 'Wentii'</t>
+          <t>Alocasia 'Pink Dragon'</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -791,16 +787,16 @@
         <v>1</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1820</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Alocasia amazonica poly var</t>
+          <t>Alocasia 'Portora'</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -812,16 +808,16 @@
         <v>1</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>4420</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Baginda 'Silver Dragon'</t>
+          <t>Alocasia 'Wentii'</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -833,16 +829,16 @@
         <v>1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>520</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Alocasia baginda Dragon Scale var</t>
+          <t>Alocasia 'Yucatan Princess' pink</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -854,16 +850,16 @@
         <v>1</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>5200</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Betwing</t>
+          <t>Alocasia 'Yucatan Princess' pink variegata</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -875,16 +871,16 @@
         <v>1</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>312</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Bisma Platinum</t>
+          <t>Alocasia amazonica poly variegata</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -896,16 +892,16 @@
         <v>1</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>312</v>
+        <v>4420</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Alocasia black Velvet pink variegata</t>
+          <t>Alocasia baginda 'Dragon Scale' aurea</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -917,16 +913,16 @@
         <v>1</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>6240</v>
+        <v>4420</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Alocasia chanterii pink variegata</t>
+          <t>Alocasia Baginda 'Silver Dragon'</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -938,16 +934,16 @@
         <v>1</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>5200</v>
+        <v>520</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Alocasia chantrieri var</t>
+          <t>Alocasia baginda Dragon Scale variegata</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -968,7 +964,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Alocasia cucullata</t>
+          <t>Alocasia Bat Wing</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -980,16 +976,16 @@
         <v>1</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>780</v>
+        <v>312</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Alocasia cuprea pink variegata</t>
+          <t>Alocasia Bisma Platinum</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1001,16 +997,16 @@
         <v>1</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>700</v>
+        <v>6</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>36400</v>
+        <v>312</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Alocasia dragon scale albo</t>
+          <t>Alocasia black Velvet pink variegata</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1022,16 +1018,16 @@
         <v>1</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>5200</v>
+        <v>6240</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Alocasia dragon scale variegata</t>
+          <t>Alocasia chantrieri pink variegata</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1052,7 +1048,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Frydek var white</t>
+          <t>Alocasia chantrieri variegata</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1064,16 +1060,16 @@
         <v>1</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>3380</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Frydek var.</t>
+          <t>Alocasia cucullata</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1085,16 +1081,16 @@
         <v>1</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>3380</v>
+        <v>780</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Gageana Aurea</t>
+          <t>Alocasia cuprea pink variegata</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1106,16 +1102,16 @@
         <v>1</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>65</v>
+        <v>700</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>3380</v>
+        <v>36400</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Alocasia gageana var</t>
+          <t>Alocasia dragon scale albo</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1127,16 +1123,16 @@
         <v>1</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>3380</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Heart Ballon var</t>
+          <t>Alocasia dragon scale variegata</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1148,16 +1144,16 @@
         <v>1</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>6760</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Maharani Albo</t>
+          <t>Alocasia Frydek variegata</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1169,16 +1165,16 @@
         <v>1</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>7800</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Melo Albo</t>
+          <t>Alocasia Frydek variegata white</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1190,16 +1186,16 @@
         <v>1</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>250</v>
+        <v>65</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>13000</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Alocasia odora variegated Batik</t>
+          <t>Alocasia Gageana Aurea</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1211,16 +1207,16 @@
         <v>1</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>120</v>
+        <v>65</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>6240</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Plaminggiana</t>
+          <t>Alocasia gageana variegata</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1232,16 +1228,16 @@
         <v>1</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>312</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Psuedo sanderian a Pink Variegated</t>
+          <t>Alocasia Maharani Albo</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1252,13 +1248,17 @@
       <c r="C38" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="5" t="n"/>
+      <c r="D38" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>7800</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Alocasia sanderiana 'Nobilis'</t>
+          <t>Alocasia Melo Albo</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1270,16 +1270,16 @@
         <v>1</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>10400</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Alocasia scalperum</t>
+          <t>Alocasia odora 'Batik' variegated</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1291,16 +1291,16 @@
         <v>1</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>520</v>
+        <v>6240</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Scalprum var white</t>
+          <t>Alocasia plumbea</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1312,16 +1312,16 @@
         <v>1</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>450</v>
+        <v>6</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>23400</v>
+        <v>312</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Alocasia silver albo</t>
+          <t>Alocasia pseudosanderiana pink variegated</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1332,17 +1332,13 @@
       <c r="C42" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="E42" s="5" t="n">
-        <v>13000</v>
-      </c>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Silver Dragon Albo</t>
+          <t>Alocasia sanderiana 'Nobilis'</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -1354,16 +1350,16 @@
         <v>1</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>13000</v>
+        <v>10400</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Sulver Dragon</t>
+          <t>Alocasia scalprum</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1375,16 +1371,16 @@
         <v>1</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>780</v>
+        <v>520</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Alocasia variegated mahrani albo</t>
+          <t>Alocasia Scalprum variegata white</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1396,16 +1392,16 @@
         <v>1</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>150</v>
+        <v>450</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>7800</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Yucatan Pink</t>
+          <t>Alocasia silver albo</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1417,16 +1413,16 @@
         <v>1</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>4680</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Alocasia Yucatan pink variegata</t>
+          <t>Alocasia Silver Dragon</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1438,16 +1434,16 @@
         <v>1</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>5200</v>
+        <v>780</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Alocasia ’Helian‘</t>
+          <t>Alocasia Silver Dragon Albo</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1458,13 +1454,17 @@
       <c r="C48" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="5" t="n"/>
+      <c r="D48" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>13000</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Dragon scale aurea</t>
+          <t>Alocasia variegated Maharani albo</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -1476,16 +1476,16 @@
         <v>1</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>85</v>
+        <v>150</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>4420</v>
+        <v>7800</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Anthurium ace of spades X papillilaminum</t>
+          <t>Anthurium 'BVIT'</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1496,13 +1496,17 @@
       <c r="C50" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="5" t="n"/>
+      <c r="D50" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>2340</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Anthurium black emerald x michelle</t>
+          <t>Anthurium 'Dorayaki'</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -1514,16 +1518,16 @@
         <v>1</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>2600</v>
+        <v>364</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Anthurium bloody night x DP</t>
+          <t>Anthurium 'Peitchi'</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1535,16 +1539,16 @@
         <v>1</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>2340</v>
+        <v>260</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Bvit</t>
+          <t>Anthurium 'Red Tiger' x 'Zara Michelle'</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -1556,16 +1560,16 @@
         <v>1</v>
       </c>
       <c r="D53" s="4" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>2340</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Carla blackiae valora</t>
+          <t>Anthurium ace of spades X papillilaminum</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1576,17 +1580,13 @@
       <c r="C54" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D54" s="4" t="n">
-        <v>90</v>
-      </c>
-      <c r="E54" s="5" t="n">
-        <v>4680</v>
-      </c>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Carla x Bvep</t>
+          <t>Anthurium black emerald x michelle</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -1598,16 +1598,16 @@
         <v>1</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>4160</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Anthurium clarinervium</t>
+          <t>Anthurium bloody night x DP</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1619,16 +1619,16 @@
         <v>1</v>
       </c>
       <c r="D56" s="4" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>2080</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Clarinerviumhybrid sulanjana</t>
+          <t>Anthurium Carla blackiae valora</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -1640,16 +1640,16 @@
         <v>1</v>
       </c>
       <c r="D57" s="4" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>2080</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Anthurium crystallinum</t>
+          <t>Anthurium Carla x Bvep</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -1661,16 +1661,16 @@
         <v>1</v>
       </c>
       <c r="D58" s="4" t="n">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>364</v>
+        <v>4160</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Anthurium crystallinum Hope × Anthurium magnificum</t>
+          <t>Anthurium clarinervium</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -1682,16 +1682,16 @@
         <v>1</v>
       </c>
       <c r="D59" s="4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>1820</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Dark Handsome</t>
+          <t>Anthurium clarinervium hybrid 'Sulanjana'</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -1703,16 +1703,16 @@
         <v>1</v>
       </c>
       <c r="D60" s="4" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>5200</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Dockblok x Michelle</t>
+          <t>Anthurium crystallinum</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -1724,16 +1724,16 @@
         <v>1</v>
       </c>
       <c r="D61" s="4" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>1560</v>
+        <v>364</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Doroyaki</t>
+          <t>Anthurium crystallinum Hope x Anthurium magnificum</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -1745,16 +1745,16 @@
         <v>1</v>
       </c>
       <c r="D62" s="4" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>364</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Dressleri x mystiq</t>
+          <t>Anthurium Dark Handsome</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -1766,16 +1766,16 @@
         <v>1</v>
       </c>
       <c r="D63" s="4" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>4680</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Anthurium hybrid DocBlock</t>
+          <t>Anthurium Dockblok x Michelle</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -1787,16 +1787,16 @@
         <v>1</v>
       </c>
       <c r="D64" s="4" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>2080</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Lucu x mystiq</t>
+          <t>Anthurium Dressleri x mystiq</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -1808,16 +1808,16 @@
         <v>1</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>2080</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Anthurium luxurians</t>
+          <t>Anthurium hybrid DocBlock</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -1829,16 +1829,16 @@
         <v>1</v>
       </c>
       <c r="D66" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>1300</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Anthurium michelle x Zara michelle</t>
+          <t>Anthurium Lucu x mystiq</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -1850,16 +1850,16 @@
         <v>1</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1300</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Anthurium modeanum</t>
+          <t>Anthurium luxurians</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -1871,16 +1871,16 @@
         <v>1</v>
       </c>
       <c r="D68" s="4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>780</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Anthurium mystiq mutation</t>
+          <t>Anthurium michelle x Zara michelle</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -1892,16 +1892,16 @@
         <v>1</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>2600</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Night Dragon</t>
+          <t>Anthurium moodeanum</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -1913,16 +1913,16 @@
         <v>1</v>
       </c>
       <c r="D70" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>5200</v>
+        <v>780</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Papi black stone</t>
+          <t>Anthurium mystiq mutation</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -1934,16 +1934,16 @@
         <v>1</v>
       </c>
       <c r="D71" s="4" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="E71" s="5" t="n">
-        <v>4680</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Papi x Bassae</t>
+          <t>Anthurium Night Dragon</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -1955,16 +1955,16 @@
         <v>1</v>
       </c>
       <c r="D72" s="4" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>312</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Papi x Zara michelle</t>
+          <t>Anthurium Papi black stone</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -1985,7 +1985,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Peitchi</t>
+          <t>Anthurium Papi x Bassae</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -1997,16 +1997,16 @@
         <v>1</v>
       </c>
       <c r="D74" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E74" s="5" t="n">
-        <v>260</v>
+        <v>312</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Anthurium poldipolium</t>
+          <t>Anthurium Papi x Zara michelle</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -2018,16 +2018,16 @@
         <v>1</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="E75" s="5" t="n">
-        <v>3380</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Red spider</t>
+          <t>Anthurium podophyllum</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2039,16 +2039,16 @@
         <v>1</v>
       </c>
       <c r="D76" s="4" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>4680</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Red Tiger</t>
+          <t>Anthurium Red spider</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2060,16 +2060,16 @@
         <v>1</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="E77" s="5" t="n">
-        <v>624</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Red x Lucu</t>
+          <t>Anthurium Red Tiger</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2081,16 +2081,16 @@
         <v>1</v>
       </c>
       <c r="D78" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E78" s="5" t="n">
-        <v>416</v>
+        <v>624</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Anthurium regale × Anthurium magnificum × Anthurium clarinervium</t>
+          <t>Anthurium Red x Lucu</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -2102,16 +2102,16 @@
         <v>1</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E79" s="5" t="n">
-        <v>1820</v>
+        <v>416</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Anthurium RVDP x michelle</t>
+          <t>Anthurium regale x Anthurium magnificum x Anthurium clarinervium</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2123,16 +2123,16 @@
         <v>1</v>
       </c>
       <c r="D80" s="4" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E80" s="5" t="n">
-        <v>1560</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Wendlingeri</t>
+          <t>Anthurium RVDP x michelle</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -2144,16 +2144,16 @@
         <v>1</v>
       </c>
       <c r="D81" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E81" s="5" t="n">
-        <v>3120</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Anthurium Zara Michelle</t>
+          <t>Anthurium Wendlingeri</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2165,16 +2165,16 @@
         <v>1</v>
       </c>
       <c r="D82" s="4" t="n">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="E82" s="5" t="n">
-        <v>832</v>
+        <v>3120</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Red Tiger x Zara Michelle</t>
+          <t>Anthurium Zara Michelle</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -2186,16 +2186,16 @@
         <v>1</v>
       </c>
       <c r="D83" s="4" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E83" s="5" t="n">
-        <v>1820</v>
+        <v>832</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Begonia mocca</t>
+          <t>Begonia (mixed varieties)</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2207,16 +2207,16 @@
         <v>1</v>
       </c>
       <c r="D84" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E84" s="5" t="n">
-        <v>520</v>
+        <v>104</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Begonia Red silver</t>
+          <t>Begonia mocca</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Begonia Rex motherplan</t>
+          <t>Begonia Polka Dot</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2249,16 +2249,16 @@
         <v>1</v>
       </c>
       <c r="D86" s="4" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E86" s="5" t="n">
-        <v>1300</v>
+        <v>520</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Begonia volkadot</t>
+          <t>Begonia Red silver</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -2279,7 +2279,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Begonian semua jenis</t>
+          <t>Begonia rex (mother plant)</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2291,10 +2291,10 @@
         <v>1</v>
       </c>
       <c r="D88" s="4" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E88" s="5" t="n">
-        <v>104</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="89">
@@ -2405,7 +2405,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Calathea 'Green Beauty'</t>
+          <t>Calathea 'C063'</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -2417,16 +2417,16 @@
         <v>1</v>
       </c>
       <c r="D94" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E94" s="5" t="n">
-        <v>624</v>
+        <v>780</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Calathea 'Purple Rainbow'</t>
+          <t>Calathea 'Green Beauty'</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Calathea 'Rosy'</t>
+          <t>Calathea 'Purple Rainbow'</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -2468,7 +2468,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Calathea 'Water color'</t>
+          <t>Calathea 'Rosy'</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -2480,16 +2480,16 @@
         <v>1</v>
       </c>
       <c r="D97" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E97" s="5" t="n">
-        <v>780</v>
+        <v>624</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Calathea bella</t>
+          <t>Calathea 'Water color'</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -2510,7 +2510,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Calathea C063</t>
+          <t>Calathea bella</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -2762,7 +2762,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Calathea picturata "Crimson"</t>
+          <t>Calathea picturata 'Crimson'</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Calathea warszewiczii</t>
+          <t>Calathea warscewiczii</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -2951,7 +2951,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Cordyline 'Pink Champion'</t>
+          <t>Cordyline 'Giant Blizzard'</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -2963,16 +2963,16 @@
         <v>1</v>
       </c>
       <c r="D120" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E120" s="5" t="n">
-        <v>520</v>
+        <v>780</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Cordyline australis 'Red Sensation'</t>
+          <t>Cordyline 'Pink Champion'</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -2993,7 +2993,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Cordyline australis 'Red Star'</t>
+          <t>Cordyline australis 'Red Sensation'</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3014,7 +3014,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Cordyline giganteum 'blizzard'</t>
+          <t>Cordyline australis 'Red Star'</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -3026,10 +3026,10 @@
         <v>1</v>
       </c>
       <c r="D123" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E123" s="5" t="n">
-        <v>780</v>
+        <v>520</v>
       </c>
     </row>
     <row r="124">
@@ -3182,7 +3182,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Dieffenbachia 'Sterling'</t>
+          <t>Dieffenbachia 'Avocado'</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -3203,7 +3203,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Dieffenbachia 'Tropic Marianne'</t>
+          <t>Dieffenbachia 'Sterling'</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -3224,7 +3224,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Dieffenbachia avocado</t>
+          <t>Dieffenbachia 'Sublime'</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -3235,17 +3235,13 @@
       <c r="C133" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D133" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E133" s="5" t="n">
-        <v>364</v>
-      </c>
+      <c r="D133" s="4" t="n"/>
+      <c r="E133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Dieffenbachia maculata 'Tropical tiki'</t>
+          <t>Dieffenbachia 'Tropic Marianne'</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -3257,16 +3253,16 @@
         <v>1</v>
       </c>
       <c r="D134" s="4" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E134" s="5" t="n">
-        <v>780</v>
+        <v>364</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Dieffenbachia White blizzard</t>
+          <t>Dieffenbachia 'White Blizzard'</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -3287,7 +3283,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Dieffenbachia ’Sublime‘</t>
+          <t>Dieffenbachia maculata 'Tropical tiki'</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -3298,13 +3294,17 @@
       <c r="C136" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D136" s="4" t="n"/>
-      <c r="E136" s="5" t="n"/>
+      <c r="D136" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E136" s="5" t="n">
+        <v>780</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Domesticum</t>
+          <t>Dracaena Golden Heart</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -3316,16 +3316,16 @@
         <v>1</v>
       </c>
       <c r="D137" s="4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E137" s="5" t="n">
-        <v>104</v>
+        <v>780</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Dracaena Golden Heart</t>
+          <t>Dracaena reflexa 'Variegata'</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -3346,28 +3346,28 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Dracaena reflexa 'Variegata'</t>
+          <t>Ficus benghalensis Audrey</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Dracaena</t>
+          <t>Ficus</t>
         </is>
       </c>
       <c r="C139" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D139" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E139" s="5" t="n">
-        <v>780</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Ficus benghalensis Audrey</t>
+          <t>Ficus elastica 'Ruby'</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -3379,16 +3379,16 @@
         <v>1</v>
       </c>
       <c r="D140" s="4" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E140" s="5" t="n">
-        <v>1820</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Ficus elastica 'Ruby'</t>
+          <t>Ficus Elastica 'Shivereana'</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -3400,16 +3400,16 @@
         <v>1</v>
       </c>
       <c r="D141" s="4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E141" s="5" t="n">
-        <v>1040</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Ficus Elastica 'Shivereana'</t>
+          <t>Ficus elastica 'Tineke'</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -3421,16 +3421,16 @@
         <v>1</v>
       </c>
       <c r="D142" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E142" s="5" t="n">
-        <v>1820</v>
+        <v>780</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Ficus elastica 'Tineke'</t>
+          <t>Ficus elastica Burgundy</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -3451,7 +3451,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Ficus elastica Burgundy</t>
+          <t>Ficus lyrata</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -3463,16 +3463,16 @@
         <v>1</v>
       </c>
       <c r="D144" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E144" s="5" t="n">
-        <v>780</v>
+        <v>624</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Ficus lyrata</t>
+          <t>Ficus lyrata 'Bambino'</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -3493,7 +3493,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Ficus lyrata 'Bambino'</t>
+          <t>Ficus lyrata cv.</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -3514,33 +3514,33 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Ficus lyrata cv.</t>
+          <t>Hoya australis Lisa</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Ficus</t>
+          <t>Hoya</t>
         </is>
       </c>
       <c r="C147" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D147" s="4" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E147" s="5" t="n">
-        <v>624</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Flobe x Mayoy</t>
+          <t>Hoya bencalensis splash</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Ficus</t>
+          <t>Hoya</t>
         </is>
       </c>
       <c r="C148" s="3" t="n">
@@ -3556,28 +3556,28 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Glorosium Dark Foam</t>
+          <t>Hoya black cat</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Ficus</t>
+          <t>Hoya</t>
         </is>
       </c>
       <c r="C149" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D149" s="4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E149" s="5" t="n">
-        <v>260</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Haderasium</t>
+          <t>Hoya carnosa Madara snow angel</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -3589,16 +3589,16 @@
         <v>1</v>
       </c>
       <c r="D150" s="4" t="n">
-        <v>40</v>
+        <v>300</v>
       </c>
       <c r="E150" s="5" t="n">
-        <v>2080</v>
+        <v>15600</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Hoya australis Lisa</t>
+          <t>Hoya caudata</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -3619,7 +3619,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Hoya bencai splash</t>
+          <t>Hoya crassipetiolata variegata</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -3631,16 +3631,16 @@
         <v>1</v>
       </c>
       <c r="D152" s="4" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E152" s="5" t="n">
-        <v>2340</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Hoya black cat</t>
+          <t>Hoya Kapuas</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -3652,16 +3652,16 @@
         <v>1</v>
       </c>
       <c r="D153" s="4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E153" s="5" t="n">
-        <v>1040</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Hoya carnosa Madara snow angel</t>
+          <t>Hoya latifolia Sarawak silver</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -3673,16 +3673,16 @@
         <v>1</v>
       </c>
       <c r="D154" s="4" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="E154" s="5" t="n">
-        <v>15600</v>
+        <v>10400</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Hoya caudata</t>
+          <t>Hoya mitrata kapuas silver</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -3694,16 +3694,16 @@
         <v>1</v>
       </c>
       <c r="D155" s="4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E155" s="5" t="n">
-        <v>1040</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Hoya crassipeteolata variegata</t>
+          <t>Hoya sigillatis splash</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -3715,16 +3715,16 @@
         <v>1</v>
       </c>
       <c r="D156" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E156" s="5" t="n">
-        <v>1040</v>
+        <v>832</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Hoya Kapuas</t>
+          <t>Hoya sp. (Haderasium)</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -3736,16 +3736,16 @@
         <v>1</v>
       </c>
       <c r="D157" s="4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E157" s="5" t="n">
-        <v>1820</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Hoya latifolia Sarawak silver</t>
+          <t>Hoya sp. kapuas</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -3757,84 +3757,84 @@
         <v>1</v>
       </c>
       <c r="D158" s="4" t="n">
-        <v>200</v>
+        <v>45</v>
       </c>
       <c r="E158" s="5" t="n">
-        <v>10400</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Hoya mitrata kapuas silver</t>
+          <t>Jewel orchid 'Jose Buono'</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Hoya</t>
+          <t>Jewel orchid</t>
         </is>
       </c>
       <c r="C159" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D159" s="4" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E159" s="5" t="n">
-        <v>1820</v>
+        <v>208</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Hoya Sigilatis splash</t>
+          <t>Jewel orchid 'Koreaseus'</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Hoya</t>
+          <t>Jewel orchid</t>
         </is>
       </c>
       <c r="C160" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D160" s="4" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E160" s="5" t="n">
-        <v>832</v>
+        <v>208</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Hoya sp kapuas</t>
+          <t>Jewel orchid 'Mega Sperma'</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Hoya</t>
+          <t>Jewel orchid</t>
         </is>
       </c>
       <c r="C161" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D161" s="4" t="n">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="E161" s="5" t="n">
-        <v>2340</v>
+        <v>208</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Jewel Cystorchis</t>
+          <t>Jewel orchid (green)</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Jewel orchid</t>
         </is>
       </c>
       <c r="C162" s="3" t="n">
@@ -3850,12 +3850,12 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Jewel Green Orchid</t>
+          <t>Jewel orchid (red)</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Jewel orchid</t>
         </is>
       </c>
       <c r="C163" s="3" t="n">
@@ -3871,12 +3871,12 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Jewel Red Orchid</t>
+          <t>Jewel orchid Cystorchis</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Jewel orchid</t>
         </is>
       </c>
       <c r="C164" s="3" t="n">
@@ -3892,112 +3892,112 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Jose Buono</t>
+          <t>Maranta leuconeura 'Erythrophylla'</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Maranta</t>
         </is>
       </c>
       <c r="C165" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D165" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E165" s="5" t="n">
-        <v>208</v>
+        <v>780</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Koreaseus</t>
+          <t>Maranta Leuconeura 'Marisela'</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Maranta</t>
         </is>
       </c>
       <c r="C166" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D166" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E166" s="5" t="n">
-        <v>208</v>
+        <v>780</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Mega Sperma</t>
+          <t>Monstera 'White monster'</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Monstera</t>
         </is>
       </c>
       <c r="C167" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D167" s="4" t="n">
-        <v>4</v>
+        <v>95</v>
       </c>
       <c r="E167" s="5" t="n">
-        <v>208</v>
+        <v>4940</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Maranta leuconeura 'Erythrophylla'</t>
+          <t>Monstera adansonii</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Maranta</t>
+          <t>Monstera</t>
         </is>
       </c>
       <c r="C168" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D168" s="4" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E168" s="5" t="n">
-        <v>780</v>
+        <v>208</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Maranta Leuconeura 'Marisela'</t>
+          <t>Monstera adansonii Albo variegata</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Maranta</t>
+          <t>Monstera</t>
         </is>
       </c>
       <c r="C169" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D169" s="4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E169" s="5" t="n">
-        <v>780</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Monstera 'White monster'</t>
+          <t>Monstera adansonii jepang variegata</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -4009,16 +4009,16 @@
         <v>1</v>
       </c>
       <c r="D170" s="4" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="E170" s="5" t="n">
-        <v>4940</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Monstera adansoni</t>
+          <t>Monstera Albo variegata</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -4030,16 +4030,16 @@
         <v>1</v>
       </c>
       <c r="D171" s="4" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E171" s="5" t="n">
-        <v>208</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Monstera adansoni Albo variegata</t>
+          <t>Monstera aurea variegata</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -4060,7 +4060,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>Monstera adansoni jepang variegata</t>
+          <t>Monstera Creme Brulee</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
@@ -4071,17 +4071,13 @@
       <c r="C173" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D173" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="E173" s="5" t="n">
-        <v>1300</v>
-      </c>
+      <c r="D173" s="4" t="n"/>
+      <c r="E173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Monstera Albo variegata</t>
+          <t>Monstera Creme Brulee variegata</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -4092,17 +4088,13 @@
       <c r="C174" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D174" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="E174" s="5" t="n">
-        <v>1300</v>
-      </c>
+      <c r="D174" s="4" t="n"/>
+      <c r="E174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Monstera aurea variegata</t>
+          <t>Monstera deliciosa</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -4114,16 +4106,16 @@
         <v>1</v>
       </c>
       <c r="D175" s="4" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E175" s="5" t="n">
-        <v>1300</v>
+        <v>416</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Monstera crame brulee</t>
+          <t>Monstera deliciosa albo</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -4134,13 +4126,17 @@
       <c r="C176" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D176" s="4" t="n"/>
-      <c r="E176" s="5" t="n"/>
+      <c r="D176" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E176" s="5" t="n">
+        <v>1040</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>Monstera crame brulee variegata</t>
+          <t>Monstera deliciosa legacy</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -4157,7 +4153,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Monstera deliciosa albo</t>
+          <t>Monstera Deliciosa Variegata</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -4169,16 +4165,16 @@
         <v>1</v>
       </c>
       <c r="D178" s="4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E178" s="5" t="n">
-        <v>1040</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Monstera deliciosa legacy</t>
+          <t>Monstera karstenianum 'Peru'</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -4189,13 +4185,17 @@
       <c r="C179" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D179" s="4" t="n"/>
-      <c r="E179" s="5" t="n"/>
+      <c r="D179" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E179" s="5" t="n">
+        <v>156</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Monstera Deliciosa Variegata</t>
+          <t>Monstera Marmorata</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -4207,16 +4207,16 @@
         <v>1</v>
       </c>
       <c r="D180" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E180" s="5" t="n">
-        <v>1820</v>
+        <v>780</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Monstera Delocasia</t>
+          <t>Monstera Thai Constellation</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -4228,16 +4228,16 @@
         <v>1</v>
       </c>
       <c r="D181" s="4" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E181" s="5" t="n">
-        <v>416</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Monstera Marmorata</t>
+          <t>Monstera Variegata</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -4249,16 +4249,16 @@
         <v>1</v>
       </c>
       <c r="D182" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E182" s="5" t="n">
-        <v>780</v>
+        <v>416</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Monstera Peru Karstenianum</t>
+          <t>Monstera White Tiger</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -4270,79 +4270,75 @@
         <v>1</v>
       </c>
       <c r="D183" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E183" s="5" t="n">
-        <v>156</v>
+        <v>364</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Monstera Thai Constellation</t>
+          <t>Peperomia argyreia (Watermelon)</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Monstera</t>
+          <t>Peperomia</t>
         </is>
       </c>
       <c r="C184" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D184" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E184" s="5" t="n">
-        <v>1040</v>
+        <v>104</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Monstera Variegata</t>
+          <t>Philodendron 'Atom'</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>Monstera</t>
+          <t>Philodendron</t>
         </is>
       </c>
       <c r="C185" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D185" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E185" s="5" t="n">
-        <v>416</v>
-      </c>
+      <c r="D185" s="4" t="n"/>
+      <c r="E185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Monstera White Tiger</t>
+          <t>Philodendron 'Birkin'</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Monstera</t>
+          <t>Philodendron</t>
         </is>
       </c>
       <c r="C186" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D186" s="4" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>364</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>P. Flobe x joepii</t>
+          <t>Philodendron 'Burle Marx' Albo Variegata</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -4354,16 +4350,16 @@
         <v>1</v>
       </c>
       <c r="D187" s="4" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="E187" s="5" t="n">
-        <v>5200</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>P. Flobe x tortum</t>
+          <t>Philodendron 'El Choco Red'</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -4375,16 +4371,16 @@
         <v>1</v>
       </c>
       <c r="D188" s="4" t="n">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>4160</v>
+        <v>780</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>P. Florida beauty x bobce</t>
+          <t>Philodendron 'Florida Beauty'</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -4396,16 +4392,16 @@
         <v>1</v>
       </c>
       <c r="D189" s="4" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="E189" s="5" t="n">
-        <v>4940</v>
+        <v>520</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Phillo brandtianum</t>
+          <t>Philodendron 'Florida Beauty'</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -4417,16 +4413,16 @@
         <v>1</v>
       </c>
       <c r="D190" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E190" s="5" t="n">
-        <v>520</v>
+        <v>104</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Phillo ciapense</t>
+          <t>Philodendron 'Florida Beauty' x joepii</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -4438,16 +4434,16 @@
         <v>1</v>
       </c>
       <c r="D191" s="4" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="E191" s="5" t="n">
-        <v>936</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Phillo dark lord</t>
+          <t>Philodendron 'Florida Beauty' x mayoi</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -4459,16 +4455,16 @@
         <v>1</v>
       </c>
       <c r="D192" s="4" t="n">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="E192" s="5" t="n">
-        <v>624</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Phillo Domesticum</t>
+          <t>Philodendron 'Florida Beauty' x tortum</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -4480,16 +4476,16 @@
         <v>1</v>
       </c>
       <c r="D193" s="4" t="n">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="E193" s="5" t="n">
-        <v>364</v>
+        <v>4160</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Phillo flobe</t>
+          <t>Philodendron 'Florida Ghost'</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -4501,16 +4497,16 @@
         <v>1</v>
       </c>
       <c r="D194" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E194" s="5" t="n">
-        <v>520</v>
+        <v>156</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Phillo majesticum</t>
+          <t>Philodendron 'Gloriosum'</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -4522,16 +4518,16 @@
         <v>1</v>
       </c>
       <c r="D195" s="4" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="E195" s="5" t="n">
-        <v>624</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Phillo pink Congo</t>
+          <t>Philodendron 'Imperial Green'</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -4543,16 +4539,16 @@
         <v>1</v>
       </c>
       <c r="D196" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E196" s="5" t="n">
-        <v>624</v>
+        <v>416</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Phillo pink princes</t>
+          <t>Philodendron 'Imperial Red'</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -4564,16 +4560,16 @@
         <v>1</v>
       </c>
       <c r="D197" s="4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E197" s="5" t="n">
-        <v>936</v>
+        <v>624</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Phillo strawberry shake</t>
+          <t>Philodendron 'Moonlight'</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -4584,17 +4580,13 @@
       <c r="C198" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D198" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="E198" s="5" t="n">
-        <v>624</v>
-      </c>
+      <c r="D198" s="4" t="n"/>
+      <c r="E198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>Phillo weple way</t>
+          <t>Philodendron 'Painted Lady'</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -4605,17 +4597,13 @@
       <c r="C199" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D199" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E199" s="5" t="n">
-        <v>312</v>
-      </c>
+      <c r="D199" s="4" t="n"/>
+      <c r="E199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Phillo white knight</t>
+          <t>Philodendron 'Pink Princess' galaxy</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -4627,16 +4615,16 @@
         <v>1</v>
       </c>
       <c r="D200" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E200" s="5" t="n">
-        <v>520</v>
+        <v>156</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Anderson</t>
+          <t>Philodendron 'Pink Princess' marble</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -4648,16 +4636,16 @@
         <v>1</v>
       </c>
       <c r="D201" s="4" t="n">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="E201" s="5" t="n">
-        <v>208</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Ciapense</t>
+          <t>Philodendron 'Ring of Fire'</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -4669,16 +4657,16 @@
         <v>1</v>
       </c>
       <c r="D202" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E202" s="5" t="n">
-        <v>208</v>
+        <v>260</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Dark lord</t>
+          <t>Philodendron 'Ring of Fire'</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -4690,16 +4678,16 @@
         <v>1</v>
       </c>
       <c r="D203" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E203" s="5" t="n">
-        <v>208</v>
+        <v>260</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Domesticum</t>
+          <t>Philodendron 'White Knight'</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -4711,16 +4699,16 @@
         <v>1</v>
       </c>
       <c r="D204" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E204" s="5" t="n">
-        <v>208</v>
+        <v>520</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Erubescens</t>
+          <t>Philodendron 'White Princess'</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -4732,16 +4720,16 @@
         <v>1</v>
       </c>
       <c r="D205" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E205" s="5" t="n">
-        <v>208</v>
+        <v>520</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Flobe</t>
+          <t>Philodendron 'Xanadu'</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -4752,17 +4740,13 @@
       <c r="C206" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D206" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E206" s="5" t="n">
-        <v>104</v>
-      </c>
+      <c r="D206" s="4" t="n"/>
+      <c r="E206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Haderaceum</t>
+          <t>Philodendron Anderson</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -4774,16 +4758,16 @@
         <v>1</v>
       </c>
       <c r="D207" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E207" s="5" t="n">
-        <v>260</v>
+        <v>208</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Mamey</t>
+          <t>Philodendron atabapoense pink variegata</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -4795,16 +4779,16 @@
         <v>1</v>
       </c>
       <c r="D208" s="4" t="n">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="E208" s="5" t="n">
-        <v>156</v>
+        <v>10400</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Pink Princess Marble</t>
+          <t>Philodendron billitiae variegata</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -4816,16 +4800,16 @@
         <v>1</v>
       </c>
       <c r="D209" s="4" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="E209" s="5" t="n">
-        <v>208</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Strawberry Shake</t>
+          <t>Philodendron Birkin variegated</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -4837,16 +4821,16 @@
         <v>1</v>
       </c>
       <c r="D210" s="4" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E210" s="5" t="n">
-        <v>208</v>
+        <v>3380</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron white knight</t>
+          <t>Philodendron brandtianum</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -4858,16 +4842,16 @@
         <v>1</v>
       </c>
       <c r="D211" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E211" s="5" t="n">
-        <v>208</v>
+        <v>520</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron white wijard</t>
+          <t>Philodendron caramel Marble variegata</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -4879,16 +4863,16 @@
         <v>1</v>
       </c>
       <c r="D212" s="4" t="n">
-        <v>4</v>
+        <v>95</v>
       </c>
       <c r="E212" s="5" t="n">
-        <v>208</v>
+        <v>4940</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Phillodendron Wiple Way</t>
+          <t>Philodendron ciapense</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -4900,16 +4884,16 @@
         <v>1</v>
       </c>
       <c r="D213" s="4" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E213" s="5" t="n">
-        <v>208</v>
+        <v>936</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Philo Florida Beuty</t>
+          <t>Philodendron Ciapense</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -4921,16 +4905,16 @@
         <v>1</v>
       </c>
       <c r="D214" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E214" s="5" t="n">
-        <v>156</v>
+        <v>208</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Philo pink princes galaxy</t>
+          <t>Philodendron dark lord</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -4942,16 +4926,16 @@
         <v>1</v>
       </c>
       <c r="D215" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E215" s="5" t="n">
-        <v>156</v>
+        <v>624</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Philo. Pink Princes marble</t>
+          <t>Philodendron Dark lord</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -4963,16 +4947,16 @@
         <v>1</v>
       </c>
       <c r="D216" s="4" t="n">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="E216" s="5" t="n">
-        <v>3900</v>
+        <v>208</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Philo. Rinf of fire</t>
+          <t>Philodendron domesticum</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -4984,16 +4968,16 @@
         <v>1</v>
       </c>
       <c r="D217" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E217" s="5" t="n">
-        <v>260</v>
+        <v>104</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Atom'</t>
+          <t>Philodendron domesticum</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -5004,13 +4988,17 @@
       <c r="C218" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D218" s="4" t="n"/>
-      <c r="E218" s="5" t="n"/>
+      <c r="D218" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E218" s="5" t="n">
+        <v>364</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Birkin'</t>
+          <t>Philodendron domesticum</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -5022,16 +5010,16 @@
         <v>1</v>
       </c>
       <c r="D219" s="4" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E219" s="5" t="n">
-        <v>1560</v>
+        <v>208</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Burle Marx' Albo Variegata</t>
+          <t>Philodendron domesticum variegata</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -5043,16 +5031,16 @@
         <v>1</v>
       </c>
       <c r="D220" s="4" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="E220" s="5" t="n">
-        <v>2340</v>
+        <v>520</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Florida Ghost'</t>
+          <t>Philodendron dragon variegata</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -5064,16 +5052,16 @@
         <v>1</v>
       </c>
       <c r="D221" s="4" t="n">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="E221" s="5" t="n">
-        <v>156</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Gloriosum'</t>
+          <t>Philodendron Erubescens</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -5085,16 +5073,16 @@
         <v>1</v>
       </c>
       <c r="D222" s="4" t="n">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="E222" s="5" t="n">
-        <v>3900</v>
+        <v>208</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Imperial Green'</t>
+          <t>Philodendron Florida Beauty</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -5106,16 +5094,16 @@
         <v>1</v>
       </c>
       <c r="D223" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E223" s="5" t="n">
-        <v>416</v>
+        <v>156</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Imperial Red'</t>
+          <t>Philodendron Florida beauty x bobce</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -5127,16 +5115,16 @@
         <v>1</v>
       </c>
       <c r="D224" s="4" t="n">
-        <v>12</v>
+        <v>95</v>
       </c>
       <c r="E224" s="5" t="n">
-        <v>624</v>
+        <v>4940</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Moonlight'</t>
+          <t>Philodendron giganteum 'blizzard'</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -5147,13 +5135,17 @@
       <c r="C225" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D225" s="4" t="n"/>
-      <c r="E225" s="5" t="n"/>
+      <c r="D225" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E225" s="5" t="n">
+        <v>1820</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Painted Lady'</t>
+          <t>Philodendron gloriosum 'Dark Form'</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -5164,13 +5156,17 @@
       <c r="C226" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D226" s="4" t="n"/>
-      <c r="E226" s="5" t="n"/>
+      <c r="D226" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E226" s="5" t="n">
+        <v>260</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Ring of Fire'</t>
+          <t>Philodendron gloriosum tricolor variegata</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -5182,16 +5178,16 @@
         <v>1</v>
       </c>
       <c r="D227" s="4" t="n">
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="E227" s="5" t="n">
-        <v>260</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'White Knight '</t>
+          <t>Philodendron Gloriosum variegata</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -5203,16 +5199,16 @@
         <v>1</v>
       </c>
       <c r="D228" s="4" t="n">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="E228" s="5" t="n">
-        <v>520</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'White Princess'</t>
+          <t>Philodendron goeldii</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -5224,16 +5220,16 @@
         <v>1</v>
       </c>
       <c r="D229" s="4" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E229" s="5" t="n">
-        <v>520</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Philodendron 'Xanadu'</t>
+          <t>Philodendron goeldii spp. variegated</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -5244,13 +5240,17 @@
       <c r="C230" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D230" s="4" t="n"/>
-      <c r="E230" s="5" t="n"/>
+      <c r="D230" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="E230" s="5" t="n">
+        <v>7800</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Philodendron atabapoense pink variegata</t>
+          <t>Philodendron Green Congo hybrid</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -5262,16 +5262,16 @@
         <v>1</v>
       </c>
       <c r="D231" s="4" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="E231" s="5" t="n">
-        <v>10400</v>
+        <v>4940</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Philodendron billitiae var</t>
+          <t>Philodendron hederaceum</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -5283,16 +5283,16 @@
         <v>1</v>
       </c>
       <c r="D232" s="4" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="E232" s="5" t="n">
-        <v>5200</v>
+        <v>260</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Birkin variegated</t>
+          <t>Philodendron majesticum</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -5304,16 +5304,16 @@
         <v>1</v>
       </c>
       <c r="D233" s="4" t="n">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="E233" s="5" t="n">
-        <v>3380</v>
+        <v>624</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Philodendron caramel Marble var</t>
+          <t>Philodendron Mamey</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -5325,16 +5325,16 @@
         <v>1</v>
       </c>
       <c r="D234" s="4" t="n">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E234" s="5" t="n">
-        <v>4940</v>
+        <v>156</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Philodendron domesticum variegata</t>
+          <t>Philodendron micans variegata</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -5346,16 +5346,16 @@
         <v>1</v>
       </c>
       <c r="D235" s="4" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="E235" s="5" t="n">
-        <v>520</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Philodendron dragon variegata</t>
+          <t>Philodendron panduriforme</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -5366,17 +5366,13 @@
       <c r="C236" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D236" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="E236" s="5" t="n">
-        <v>3900</v>
-      </c>
+      <c r="D236" s="4" t="n"/>
+      <c r="E236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Philodendron EI choco red</t>
+          <t>Philodendron paraiso verde</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -5397,7 +5393,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Philodendron giganteum 'blizzard '</t>
+          <t>Philodendron pink Congo</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -5409,16 +5405,16 @@
         <v>1</v>
       </c>
       <c r="D238" s="4" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E238" s="5" t="n">
-        <v>1820</v>
+        <v>624</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Gloriosum Var.</t>
+          <t>Philodendron pink Princess</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -5430,16 +5426,16 @@
         <v>1</v>
       </c>
       <c r="D239" s="4" t="n">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="E239" s="5" t="n">
-        <v>3900</v>
+        <v>936</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Philodendron gloriousum tricollor variegata</t>
+          <t>Philodendron Pink Princess Marble</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -5451,16 +5447,16 @@
         <v>1</v>
       </c>
       <c r="D240" s="4" t="n">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="E240" s="5" t="n">
-        <v>3900</v>
+        <v>208</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Philodendron goeldii</t>
+          <t>Philodendron pink princess variegata</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -5472,16 +5468,16 @@
         <v>1</v>
       </c>
       <c r="D241" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E241" s="5" t="n">
-        <v>1040</v>
+        <v>780</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Philodendron goeldii spp variegated</t>
+          <t>Philodendron Prince of Orange</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -5493,16 +5489,16 @@
         <v>1</v>
       </c>
       <c r="D242" s="4" t="n">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="E242" s="5" t="n">
-        <v>7800</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Green Congo hybrid</t>
+          <t>Philodendron Red Congo Variegated</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -5514,16 +5510,16 @@
         <v>1</v>
       </c>
       <c r="D243" s="4" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="E243" s="5" t="n">
-        <v>4940</v>
+        <v>4420</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Philodendron micans variegata</t>
+          <t>Philodendron Red sun</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -5534,17 +5530,13 @@
       <c r="C244" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D244" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="E244" s="5" t="n">
-        <v>2340</v>
-      </c>
+      <c r="D244" s="4" t="n"/>
+      <c r="E244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Philodendron panduriforme</t>
+          <t>Philodendron sp. (Prakensis)</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -5555,13 +5547,17 @@
       <c r="C245" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D245" s="4" t="n"/>
-      <c r="E245" s="5" t="n"/>
+      <c r="D245" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E245" s="5" t="n">
+        <v>208</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>Philodendron paraiso verde</t>
+          <t>Philodendron sp. (Purbesi, Jabar)</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -5573,16 +5569,16 @@
         <v>1</v>
       </c>
       <c r="D246" s="4" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E246" s="5" t="n">
-        <v>780</v>
+        <v>468</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Philodendron pink princess variegata</t>
+          <t>Philodendron strawberry shake</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -5594,16 +5590,16 @@
         <v>1</v>
       </c>
       <c r="D247" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E247" s="5" t="n">
-        <v>780</v>
+        <v>624</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Prince of Orange</t>
+          <t>Philodendron Strawberry Shake</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -5615,16 +5611,16 @@
         <v>1</v>
       </c>
       <c r="D248" s="4" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E248" s="5" t="n">
-        <v>1560</v>
+        <v>208</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Red Congo Variegated</t>
+          <t>Philodendron tortum</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -5636,16 +5632,16 @@
         <v>1</v>
       </c>
       <c r="D249" s="4" t="n">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="E249" s="5" t="n">
-        <v>4420</v>
+        <v>780</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Red sun</t>
+          <t>Philodendron tortum variegata</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -5656,13 +5652,17 @@
       <c r="C250" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D250" s="4" t="n"/>
-      <c r="E250" s="5" t="n"/>
+      <c r="D250" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="E250" s="5" t="n">
+        <v>10400</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Philodendron tortum</t>
+          <t>Philodendron Verrucosum 'Incensi'</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -5674,16 +5674,16 @@
         <v>1</v>
       </c>
       <c r="D251" s="4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E251" s="5" t="n">
-        <v>780</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>Philodendron tortum variegata</t>
+          <t>Philodendron warscewiczii</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -5694,17 +5694,13 @@
       <c r="C252" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D252" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="E252" s="5" t="n">
-        <v>10400</v>
-      </c>
+      <c r="D252" s="4" t="n"/>
+      <c r="E252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>Philodendron Verrucosum 'Incensi'</t>
+          <t>Philodendron Whipple way</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -5716,16 +5712,16 @@
         <v>1</v>
       </c>
       <c r="D253" s="4" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E253" s="5" t="n">
-        <v>1300</v>
+        <v>312</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>Philodendron warscewiczii</t>
+          <t>Philodendron Whipple Way</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -5736,13 +5732,17 @@
       <c r="C254" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D254" s="4" t="n"/>
-      <c r="E254" s="5" t="n"/>
+      <c r="D254" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E254" s="5" t="n">
+        <v>208</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>Pilea paperomia</t>
+          <t>Philodendron white knight</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -5754,16 +5754,16 @@
         <v>1</v>
       </c>
       <c r="D255" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E255" s="5" t="n">
-        <v>104</v>
+        <v>520</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>Prakensis</t>
+          <t>Philodendron white knight</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -5784,7 +5784,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>Purbesi sp jabar</t>
+          <t>Philodendron white Wizard</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -5796,31 +5796,31 @@
         <v>1</v>
       </c>
       <c r="D257" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E257" s="5" t="n">
-        <v>468</v>
+        <v>208</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>Rhaphidophora</t>
+          <t>Pilea / Peperomia sp.</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>Philodendron</t>
+          <t>Pilea</t>
         </is>
       </c>
       <c r="C258" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D258" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E258" s="5" t="n">
-        <v>260</v>
+        <v>104</v>
       </c>
     </row>
     <row r="259">
@@ -5847,66 +5847,70 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>Schismatoglottis wallichii</t>
+          <t>Rhaphidophora sp.</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>Schismatoglottis</t>
+          <t>Rhaphidophora</t>
         </is>
       </c>
       <c r="C260" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D260" s="4" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E260" s="5" t="n">
-        <v>780</v>
+        <v>260</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>Sc. Darkcloud auera marble</t>
+          <t>Rhaphidophora tetrasperma</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus</t>
+          <t>Rhaphidophora</t>
         </is>
       </c>
       <c r="C261" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D261" s="4" t="n"/>
-      <c r="E261" s="5" t="n"/>
+      <c r="D261" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E261" s="5" t="n">
+        <v>364</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>Sc. Moonlight cloud marble</t>
+          <t>Schismatoglottis wallichii</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus</t>
+          <t>Schismatoglottis</t>
         </is>
       </c>
       <c r="C262" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D262" s="4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E262" s="5" t="n">
-        <v>1300</v>
+        <v>780</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>Sc. Rubicon GOG</t>
+          <t>Scindapsus Bakupati</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -5918,16 +5922,16 @@
         <v>1</v>
       </c>
       <c r="D263" s="4" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E263" s="5" t="n">
-        <v>1040</v>
+        <v>3120</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus Bakupati</t>
+          <t>Scindapsus Blue Albo</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -5939,16 +5943,16 @@
         <v>1</v>
       </c>
       <c r="D264" s="4" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="E264" s="5" t="n">
-        <v>3120</v>
+        <v>208</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus Blue Albo</t>
+          <t>Scindapsus Blue Salaka</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -5960,16 +5964,16 @@
         <v>1</v>
       </c>
       <c r="D265" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E265" s="5" t="n">
-        <v>208</v>
+        <v>260</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus Blue Salaka</t>
+          <t>Scindapsus Creamblue</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -5981,16 +5985,16 @@
         <v>1</v>
       </c>
       <c r="D266" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E266" s="5" t="n">
-        <v>260</v>
+        <v>104</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus Creamblue</t>
+          <t>Scindapsus Darkcloud auera marble</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
@@ -6001,12 +6005,8 @@
       <c r="C267" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D267" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E267" s="5" t="n">
-        <v>104</v>
-      </c>
+      <c r="D267" s="4" t="n"/>
+      <c r="E267" s="5" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -6074,7 +6074,7 @@
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus Silverstar</t>
+          <t>Scindapsus Moonlight cloud marble</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -6086,16 +6086,16 @@
         <v>1</v>
       </c>
       <c r="D271" s="4" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E271" s="5" t="n">
-        <v>416</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>Scindapsus Treubii</t>
+          <t>Scindapsus Rubicon GOG</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -6107,79 +6107,79 @@
         <v>1</v>
       </c>
       <c r="D272" s="4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E272" s="5" t="n">
-        <v>260</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>Spathiphyllum 'Falco'</t>
+          <t>Scindapsus Silverstar</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>Spathiphyllum</t>
+          <t>Scindapsus</t>
         </is>
       </c>
       <c r="C273" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D273" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E273" s="5" t="n">
-        <v>780</v>
+        <v>416</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>Sygnioum Tri Colour</t>
+          <t>Scindapsus Treubii</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>Syngonium</t>
+          <t>Scindapsus</t>
         </is>
       </c>
       <c r="C274" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D274" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E274" s="5" t="n">
-        <v>104</v>
+        <v>260</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>Syngonium 'Milk Confetti'</t>
+          <t>Spathiphyllum 'Falco'</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>Syngonium</t>
+          <t>Spathiphyllum</t>
         </is>
       </c>
       <c r="C275" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D275" s="4" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E275" s="5" t="n">
-        <v>208</v>
+        <v>780</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>Syngonium 'Pink'</t>
+          <t>Syngonium 'Milk Confetti'</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -6191,16 +6191,16 @@
         <v>1</v>
       </c>
       <c r="D276" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E276" s="5" t="n">
-        <v>364</v>
+        <v>208</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>Syngonium Green Splash</t>
+          <t>Syngonium 'Pink'</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -6221,7 +6221,7 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>Syngonium Milk Confetti</t>
+          <t>Syngonium Green Splash</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
@@ -6233,16 +6233,16 @@
         <v>1</v>
       </c>
       <c r="D278" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E278" s="5" t="n">
-        <v>208</v>
+        <v>364</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum 'neon'</t>
+          <t>Syngonium Milk Confetti</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
@@ -6254,16 +6254,16 @@
         <v>1</v>
       </c>
       <c r="D279" s="4" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E279" s="5" t="n">
-        <v>780</v>
+        <v>208</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum'White Buttfly'</t>
+          <t>Syngonium podophyllum 'neon'</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>Syngonium three King</t>
+          <t>Syngonium podophyllum'White Butterfly</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
@@ -6296,118 +6296,122 @@
         <v>1</v>
       </c>
       <c r="D281" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E281" s="5" t="n">
-        <v>156</v>
+        <v>780</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>ؤ integrifolia</t>
+          <t>Syngonium three King</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>Tacca</t>
+          <t>Syngonium</t>
         </is>
       </c>
       <c r="C282" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D282" s="4" t="n"/>
-      <c r="E282" s="5" t="n"/>
+      <c r="D282" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E282" s="5" t="n">
+        <v>156</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>Tetra sperma</t>
+          <t>Syngonium Tri Color</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>Tetra</t>
+          <t>Syngonium</t>
         </is>
       </c>
       <c r="C283" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D283" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E283" s="5" t="n">
-        <v>364</v>
+        <v>104</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>Watermelon Peperomia</t>
+          <t>Tacca integrifolia</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>Watermelon</t>
+          <t>Tacca</t>
         </is>
       </c>
       <c r="C284" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D284" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E284" s="5" t="n">
-        <v>104</v>
-      </c>
+      <c r="D284" s="4" t="n"/>
+      <c r="E284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>Xanthosoma lindenii</t>
+          <t>Zebrina Pink</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>Xanthosoma</t>
+          <t>Tradescantia zebrina</t>
         </is>
       </c>
       <c r="C285" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D285" s="4" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E285" s="5" t="n">
-        <v>3900</v>
+        <v>104</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>Zamya balck</t>
+          <t>Zebrina purple</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>Zamioculcas</t>
+          <t>Tradescantia zebrina</t>
         </is>
       </c>
       <c r="C286" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D286" s="4" t="n"/>
-      <c r="E286" s="5" t="n"/>
+      <c r="D286" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E286" s="5" t="n">
+        <v>156</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>Zebrina Pink</t>
+          <t>Zebrina Silver</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>Zebrina</t>
+          <t>Tradescantia zebrina</t>
         </is>
       </c>
       <c r="C287" s="3" t="n">
@@ -6423,65 +6427,61 @@
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>Zebrina purple</t>
+          <t>Zebrina White</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Zebrina</t>
+          <t>Tradescantia zebrina</t>
         </is>
       </c>
       <c r="C288" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D288" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E288" s="5" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>Zebrina Silver</t>
+          <t>Xanthosoma lindenii</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>Zebrina</t>
+          <t>Xanthosoma</t>
         </is>
       </c>
       <c r="C289" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D289" s="4" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="E289" s="5" t="n">
-        <v>104</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>Zebrina White</t>
+          <t>Zamioculcas zamiifolia (black)</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>Zebrina</t>
+          <t>Zamioculcas</t>
         </is>
       </c>
       <c r="C290" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D290" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E290" s="5" t="n">
-        <v>104</v>
-      </c>
+      <c r="D290" s="4" t="n"/>
+      <c r="E290" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E290"/>

</xml_diff>

<commit_message>
Merge Price List v22: fill missing prices, add 173-variety appendix section and Excel sheet
</commit_message>
<xml_diff>
--- a/catalog/Plant_Catalog_2026.xlsx
+++ b/catalog/Plant_Catalog_2026.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price List v22 additions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalog'!$A$1:$E$290</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Price List v22 additions'!$A$1:$G$174</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="#,##0&quot; EGP&quot;"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -77,7 +78,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -727,8 +728,12 @@
       <c r="C13" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="D13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>312</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1332,8 +1337,8 @@
       <c r="C42" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="5" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1580,8 +1585,8 @@
       <c r="C54" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="5" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3235,8 +3240,8 @@
       <c r="C133" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D133" s="4" t="n"/>
-      <c r="E133" s="5" t="n"/>
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -4071,8 +4076,8 @@
       <c r="C173" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D173" s="4" t="n"/>
-      <c r="E173" s="5" t="n"/>
+      <c r="D173" s="3" t="n"/>
+      <c r="E173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -4088,8 +4093,8 @@
       <c r="C174" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D174" s="4" t="n"/>
-      <c r="E174" s="5" t="n"/>
+      <c r="D174" s="3" t="n"/>
+      <c r="E174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -4147,8 +4152,8 @@
       <c r="C177" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D177" s="4" t="n"/>
-      <c r="E177" s="5" t="n"/>
+      <c r="D177" s="3" t="n"/>
+      <c r="E177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -4311,8 +4316,8 @@
       <c r="C185" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D185" s="4" t="n"/>
-      <c r="E185" s="5" t="n"/>
+      <c r="D185" s="3" t="n"/>
+      <c r="E185" s="3" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -4580,8 +4585,8 @@
       <c r="C198" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D198" s="4" t="n"/>
-      <c r="E198" s="5" t="n"/>
+      <c r="D198" s="3" t="n"/>
+      <c r="E198" s="3" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -4597,8 +4602,8 @@
       <c r="C199" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D199" s="4" t="n"/>
-      <c r="E199" s="5" t="n"/>
+      <c r="D199" s="3" t="n"/>
+      <c r="E199" s="3" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -4740,8 +4745,8 @@
       <c r="C206" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D206" s="4" t="n"/>
-      <c r="E206" s="5" t="n"/>
+      <c r="D206" s="3" t="n"/>
+      <c r="E206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -5366,8 +5371,8 @@
       <c r="C236" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D236" s="4" t="n"/>
-      <c r="E236" s="5" t="n"/>
+      <c r="D236" s="3" t="n"/>
+      <c r="E236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -5530,8 +5535,8 @@
       <c r="C244" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D244" s="4" t="n"/>
-      <c r="E244" s="5" t="n"/>
+      <c r="D244" s="3" t="n"/>
+      <c r="E244" s="3" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -5694,8 +5699,8 @@
       <c r="C252" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D252" s="4" t="n"/>
-      <c r="E252" s="5" t="n"/>
+      <c r="D252" s="3" t="n"/>
+      <c r="E252" s="3" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -6005,8 +6010,12 @@
       <c r="C267" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D267" s="4" t="n"/>
-      <c r="E267" s="5" t="n"/>
+      <c r="D267" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E267" s="5" t="n">
+        <v>520</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -6358,8 +6367,8 @@
       <c r="C284" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D284" s="4" t="n"/>
-      <c r="E284" s="5" t="n"/>
+      <c r="D284" s="3" t="n"/>
+      <c r="E284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -6480,11 +6489,4535 @@
       <c r="C290" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D290" s="4" t="n"/>
-      <c r="E290" s="5" t="n"/>
+      <c r="D290" s="3" t="n"/>
+      <c r="E290" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E290"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G174"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Variety</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Genus</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>USD min</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>USD max</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>EGP min</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>EGP max</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia 'Bambino'</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia 'Cuprea'</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia 'Gageana' Albo Variegata</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>8320</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>8320</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia 'Hilo Beauty'</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia 'Mickey Mouse'</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia 'Serendipity' Variegata</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>4940</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia bisma</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>312</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia cuprea 'Aurea / Caramel Latte Variegata'</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>6760</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>6760</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia gageana 'Aurea' Variegata</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia golden bone</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia longiloba</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia longiloba silver</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia low rider</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia melo</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia micholitziana 'Frydek'</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia nebula</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia regal shield</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia reginula 'Black Velvet Pink Variegata'</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>5720</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>5720</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia reginula 'Black Velvet'</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia venom</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia wentii</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia x chantrieri 'Pink Variegata'</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Alocasia</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>14560</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>14560</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium 'Aurea variegata'</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>16640</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>16640</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium 'Pink Vein'</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>4940</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium 'Purple Vein'</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>7280</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>7280</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium 'Red Crystal'</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium 'Red Crystallinum'</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>3380</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium 'Silver Blush'</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium crystallinum 'Dorayaki'</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium hybrid</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium modeanum</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium papillilaminum</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>5720</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>11440</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium papillilaminum hybrid</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>4160</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>4160</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium Purple Tiger</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium veitchii</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium waroc</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>624</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium waroc 15$</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium warocqueanum</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Anthurium</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Ardisia sp. 'Turtle Back' Pink / Purple</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Ardisia</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Begonia 'Black Fang'</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Begonia 'Brevirimosa'</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G42" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Begonia bipinnatifida</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Begonia brevirimosa subsp. exotica</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Begonia darthvaderiana</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>3380</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Begonia excoteka</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Begonia ferox</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>3380</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Begonia sillensis</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Begonia timika</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>4680</v>
+      </c>
+      <c r="G49" s="5" t="n">
+        <v>4680</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Begonia walet</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Cane-type Angel Wing Begonia hybrid</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Micro-terrarium collector Begonia</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>3120</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>3120</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Micro/Miniature Terrarium Begonia</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Rhizomatous Begonia</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G54" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Rhizomatous Bullate Begonia</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Begonia</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G55" s="5" t="n">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Caladium bicolor</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Caladium</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G56" s="5" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Caladium tikus</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Caladium</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G57" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Carica dieng / Mountain Papaya</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Carica</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="3" t="n"/>
+      <c r="E58" s="3" t="n"/>
+      <c r="F58" s="3" t="n"/>
+      <c r="G58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Carica papaya 'Dwarf'</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Carica</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F59" s="5" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Cercestis mirabilis</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Cercestis</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>312</v>
+      </c>
+      <c r="G60" s="5" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Ceropegia woodii 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Ceropegia</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F61" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G61" s="5" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Cocos nucifera var. rubescens</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Cocos</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="F62" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G62" s="5" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Colocasia esculenta 'Mojito'</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Colocasia</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F63" s="5" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Colocasia Mujito</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Colocasia</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F64" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G64" s="5" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Colocasia Mujito12$</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Colocasia</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F65" s="5" t="n">
+        <v>624</v>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Dionaea muscipula</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Dionaea</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F66" s="5" t="n">
+        <v>832</v>
+      </c>
+      <c r="G66" s="5" t="n">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Dracaena fragrans cane cuttings</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Dracaena</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F67" s="5" t="n">
+        <v>936</v>
+      </c>
+      <c r="G67" s="5" t="n">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Dracaena sanderiana</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Dracaena</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F68" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="G68" s="5" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Drimiopsis maculata</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Drimiopsis</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F69" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G69" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Echeveria agavoides varieties – Aquamarine, Bronze Beauty, Christmas, Corderoyi, Ebony, Miranda, Frank Reinelt, Prolifera, Romeo, Lipstick, Pulidonis, Romeo Rubin</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Echeveria</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="3" t="n"/>
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Euphorbia francoisii</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Euphorbia</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F71" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="G71" s="5" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Euphorbia hedyotoides</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Euphorbia</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F72" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G72" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Graptophyllum pictum 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Graptophyllum</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F73" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G73" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Homalomena rubescens 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Homalomena</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="F74" s="5" t="n">
+        <v>4160</v>
+      </c>
+      <c r="G74" s="5" t="n">
+        <v>4160</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Hoya carnosa 'Compacta Variegata'</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F75" s="5" t="n">
+        <v>1456</v>
+      </c>
+      <c r="G75" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Hoya compacta variegata</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="F76" s="5" t="n">
+        <v>1092</v>
+      </c>
+      <c r="G76" s="5" t="n">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Hoya kerii splash</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F77" s="5" t="n">
+        <v>624</v>
+      </c>
+      <c r="G77" s="5" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Hoya kerii variegata</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F78" s="5" t="n">
+        <v>676</v>
+      </c>
+      <c r="G78" s="5" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Hoya kerrii 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E79" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F79" s="5" t="n">
+        <v>3120</v>
+      </c>
+      <c r="G79" s="5" t="n">
+        <v>3120</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Hoya latifolia</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F80" s="5" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G80" s="5" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Hoya obovata variegata</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F81" s="5" t="n">
+        <v>572</v>
+      </c>
+      <c r="G81" s="5" t="n">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Hoya wayetii 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Hoya</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F82" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G82" s="5" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Labisia pumila</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Labisia</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F83" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G83" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Labisia pumila 'Pink'</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Labisia</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F84" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G84" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Monstera adansoni mint</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F85" s="5" t="n">
+        <v>468</v>
+      </c>
+      <c r="G85" s="5" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Monstera Adansoni Variegata</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F86" s="5" t="n">
+        <v>468</v>
+      </c>
+      <c r="G86" s="5" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Monstera adansonii 'Aurea' Variegata</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="F87" s="5" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G87" s="5" t="n">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Monstera adansonii variegata</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F88" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G88" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Monstera adansori mint green</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F89" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G89" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Monstera adensoni albo varigata</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F90" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G90" s="5" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Monstera aurea</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" s="3" t="n"/>
+      <c r="E91" s="3" t="n"/>
+      <c r="F91" s="3" t="n"/>
+      <c r="G91" s="3" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Monstera deliciosa 'Albo Borsigiana'</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="F92" s="5" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G92" s="5" t="n">
+        <v>5720</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Monstera deliciosa 'Aurea' Variegata</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="F93" s="5" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G93" s="5" t="n">
+        <v>4940</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Monstera varigata</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F94" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G94" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Monstera white Tiger marbel</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Monstera</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E95" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F95" s="5" t="n">
+        <v>624</v>
+      </c>
+      <c r="G95" s="5" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Musa 'Ae Ae'</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Musa</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="F96" s="5" t="n">
+        <v>6760</v>
+      </c>
+      <c r="G96" s="5" t="n">
+        <v>9360</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Musa 'Florida' variegata</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Musa</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E97" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="F97" s="5" t="n">
+        <v>4680</v>
+      </c>
+      <c r="G97" s="5" t="n">
+        <v>6240</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Musa 'Florida' Yellow variegata</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Musa</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="E98" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="F98" s="5" t="n">
+        <v>7280</v>
+      </c>
+      <c r="G98" s="5" t="n">
+        <v>7280</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Musa 'NoNo'</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Musa</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F99" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G99" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Musa acuminata 'Red Dacca'</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Musa</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F100" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G100" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Musa acuminata 'Siam Ruby'</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Musa</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="E101" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="F101" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G101" s="5" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Aurea</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E102" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F102" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G102" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Aurea variegata</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E103" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F103" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G103" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Banana variegata</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E104" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F104" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G104" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Black emerald x zara michelle</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" s="3" t="n"/>
+      <c r="E105" s="3" t="n"/>
+      <c r="F105" s="3" t="n"/>
+      <c r="G105" s="3" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Bloody night x dp</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="3" t="n"/>
+      <c r="E106" s="3" t="n"/>
+      <c r="F106" s="3" t="n"/>
+      <c r="G106" s="3" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Burle Marx variegata</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E107" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F107" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G107" s="5" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Carla original</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="F108" s="5" t="n">
+        <v>3432</v>
+      </c>
+      <c r="G108" s="5" t="n">
+        <v>3432</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Christmas</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E109" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F109" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G109" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Clarinervium</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" s="3" t="n"/>
+      <c r="E110" s="3" t="n"/>
+      <c r="F110" s="3" t="n"/>
+      <c r="G110" s="3" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Clarinervium kos magani</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" s="3" t="n"/>
+      <c r="E111" s="3" t="n"/>
+      <c r="F111" s="3" t="n"/>
+      <c r="G111" s="3" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Clarinervium 🔁 kos x magni</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" s="3" t="n"/>
+      <c r="E112" s="3" t="n"/>
+      <c r="F112" s="3" t="n"/>
+      <c r="G112" s="3" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Crystallinum</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" s="3" t="n"/>
+      <c r="E113" s="3" t="n"/>
+      <c r="F113" s="3" t="n"/>
+      <c r="G113" s="3" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Docblok</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F114" s="5" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G114" s="5" t="n">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Dorayaki</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="3" t="n"/>
+      <c r="G115" s="3" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Episcia smoke white</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F116" s="5" t="n">
+        <v>312</v>
+      </c>
+      <c r="G116" s="5" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Fortile Drak From variegata Orange</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D117" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="E117" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="F117" s="5" t="n">
+        <v>4992</v>
+      </c>
+      <c r="G117" s="5" t="n">
+        <v>4992</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Gigas</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D118" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F118" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="G118" s="5" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Golden bonee</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D119" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F119" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G119" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Jewel Cystorchis</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F120" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="G120" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Kos rc x Angel Dreams</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D121" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E121" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="F121" s="5" t="n">
+        <v>1092</v>
+      </c>
+      <c r="G121" s="5" t="n">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Lotus mini</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" s="3" t="n"/>
+      <c r="E122" s="3" t="n"/>
+      <c r="F122" s="3" t="n"/>
+      <c r="G122" s="3" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Lotus mix isi 10</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D123" s="3" t="n"/>
+      <c r="E123" s="3" t="n"/>
+      <c r="F123" s="3" t="n"/>
+      <c r="G123" s="3" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Luxurians</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="3" t="n"/>
+      <c r="E124" s="3" t="n"/>
+      <c r="F124" s="3" t="n"/>
+      <c r="G124" s="3" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Mahkota</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" s="3" t="n"/>
+      <c r="E125" s="3" t="n"/>
+      <c r="F125" s="3" t="n"/>
+      <c r="G125" s="3" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Michelle x Angel Dreams</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F126" s="5" t="n">
+        <v>2496</v>
+      </c>
+      <c r="G126" s="5" t="n">
+        <v>2496</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Milk Confetti tricolor</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E127" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F127" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G127" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Papi x Magni</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="E128" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="F128" s="5" t="n">
+        <v>2652</v>
+      </c>
+      <c r="G128" s="5" t="n">
+        <v>2652</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Paraiso Verde</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E129" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F129" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G129" s="5" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Pink princess galaxy</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E130" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F130" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G130" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Purple tiger x Michelle</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="E131" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="F131" s="5" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G131" s="5" t="n">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Red Ghost x Luxury</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="F132" s="5" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G132" s="5" t="n">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Red Tiger</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
+      <c r="F133" s="3" t="n"/>
+      <c r="G133" s="3" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Red Tiger Original Purple Serat Cakep Semi Induk</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="E134" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="F134" s="5" t="n">
+        <v>8112</v>
+      </c>
+      <c r="G134" s="5" t="n">
+        <v>8112</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Red Tiger Purple Character Purple Serat Teran</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E135" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F135" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="G135" s="5" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>RVDP x Michelle</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" s="3" t="n"/>
+      <c r="E136" s="3" t="n"/>
+      <c r="F136" s="3" t="n"/>
+      <c r="G136" s="3" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Silver dragon</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E137" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F137" s="5" t="n">
+        <v>416</v>
+      </c>
+      <c r="G137" s="5" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>String of heart</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" s="3" t="n"/>
+      <c r="E138" s="3" t="n"/>
+      <c r="F138" s="3" t="n"/>
+      <c r="G138" s="3" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Veitchii</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" s="3" t="n"/>
+      <c r="E139" s="3" t="n"/>
+      <c r="F139" s="3" t="n"/>
+      <c r="G139" s="3" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Warocqueanum</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E140" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F140" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G140" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Water Lily</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" s="3" t="n"/>
+      <c r="E141" s="3" t="n"/>
+      <c r="F141" s="3" t="n"/>
+      <c r="G141" s="3" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Zara michelle</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" s="3" t="n"/>
+      <c r="E142" s="3" t="n"/>
+      <c r="F142" s="3" t="n"/>
+      <c r="G142" s="3" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Zebrina nanouk</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Other / hybrids</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E143" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F143" s="5" t="n">
+        <v>208</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Peperomia argyreia 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Peperomia</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F144" s="5" t="n">
+        <v>1560</v>
+      </c>
+      <c r="G144" s="5" t="n">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Peperomia belimbing</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Peperomia</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E145" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F145" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G145" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Peperomia prostrata</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Peperomia</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E146" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F146" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="G146" s="5" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron 'Caramel Marble'</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="E147" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="F147" s="5" t="n">
+        <v>6760</v>
+      </c>
+      <c r="G147" s="5" t="n">
+        <v>6760</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron 'Green Congo' variegata</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D148" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E148" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F148" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G148" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron billietiae</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="E149" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="F149" s="5" t="n">
+        <v>7800</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>7800</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron Congo hybrid</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E150" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="F150" s="5" t="n">
+        <v>728</v>
+      </c>
+      <c r="G150" s="5" t="n">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron erubescens 'Strawberry Shake'</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="E151" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="F151" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron gigas</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E152" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F152" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G152" s="5" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron hederaceum var. hederaceum 'Micans' Variegata</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="E153" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="F153" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G153" s="5" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron True Pink Micans</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Philodendron</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E154" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F154" s="5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="G154" s="5" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>Pilea peperomioides</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Pilea</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E155" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F155" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G155" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Plinia cauliflora</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Plinia</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E156" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F156" s="5" t="n">
+        <v>3380</v>
+      </c>
+      <c r="G156" s="5" t="n">
+        <v>3380</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Schismatoglottis calyptrata 'Silver Stripe'</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Schismatoglottis</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E157" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F157" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G157" s="5" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Scindapsus hederaceus 'Variegata'</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Scindapsus</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="E158" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F158" s="5" t="n">
+        <v>3640</v>
+      </c>
+      <c r="G158" s="5" t="n">
+        <v>3640</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Sonerila sp. 'Purple White Vein'</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Sonerila</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E159" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F159" s="5" t="n">
+        <v>1456</v>
+      </c>
+      <c r="G159" s="5" t="n">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>ID Syngonium Dwarf Princess/Mini Christmas</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" s="3" t="n"/>
+      <c r="E160" s="3" t="n"/>
+      <c r="F160" s="3" t="n"/>
+      <c r="G160" s="3" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Deep Pink Splash</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E161" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F161" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G161" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Liliter</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" s="3" t="n"/>
+      <c r="E162" s="3" t="n"/>
+      <c r="F162" s="3" t="n"/>
+      <c r="G162" s="3" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Mango Alution</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" s="3" t="n"/>
+      <c r="E163" s="3" t="n"/>
+      <c r="F163" s="3" t="n"/>
+      <c r="G163" s="3" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Mojito</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E164" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F164" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G164" s="5" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Panda</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E165" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F165" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G165" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Pink on Pink</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D166" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E166" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F166" s="5" t="n">
+        <v>364</v>
+      </c>
+      <c r="G166" s="5" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium Pink Panda</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E167" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F167" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G167" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium podophyllum 'Red Spot Tricolor'</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D168" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E168" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="F168" s="5" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G168" s="5" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium redspot 3 colour</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E169" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F169" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="G169" s="5" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium strawberry ice</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" s="3" t="n"/>
+      <c r="E170" s="3" t="n"/>
+      <c r="F170" s="3" t="n"/>
+      <c r="G170" s="3" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium tricolor</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Syngonium</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E171" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F171" s="5" t="n">
+        <v>208</v>
+      </c>
+      <c r="G171" s="5" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>Live Cushion Moss / Pillow Moss</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Terrarium &amp; moss</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E172" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F172" s="5" t="n">
+        <v>832</v>
+      </c>
+      <c r="G172" s="5" t="n">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>Live Sheet Moss / Carpet Moss</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>Terrarium &amp; moss</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E173" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F173" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="G173" s="5" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>Thaumatophyllum warscewiczii</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Thaumatophyllum</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E174" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F174" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G174" s="5" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G174"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add reference photos for uncovered varieties, photo credits page, Photo column in Excel
</commit_message>
<xml_diff>
--- a/catalog/Plant_Catalog_2026.xlsx
+++ b/catalog/Plant_Catalog_2026.xlsx
@@ -454,7 +454,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
@@ -8550,7 +8550,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
@@ -10798,7 +10798,7 @@
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
@@ -11342,7 +11342,7 @@
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -12286,7 +12286,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>

</xml_diff>